<commit_message>
last minute updated midterms
</commit_message>
<xml_diff>
--- a/kadai/week08/midterms.xlsx
+++ b/kadai/week08/midterms.xlsx
@@ -329,12 +329,12 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>1254510229</t>
+          <t>1254510154</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>岩田　知機（イワタ　チキ）</t>
+          <t>石原　優聖（イシハラ　ユウセイ）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -355,477 +355,569 @@
       <c r="F3" s="1"/>
       <c r="G3" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 10:19</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>石原　優聖（イシハラ　ユウセイ）</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/BJkrQA9XxXABQEge
+https://toysosiki.github.io/mao01/</t>
+        </is>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3" s="1"/>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O3" s="1"/>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 経済学部 経済学科 経済</t>
+        </is>
+      </c>
+      <c r="S3" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T3" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U3" s="4" t="inlineStr">
+        <is>
+          <t>10.30.48.141</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>1254510229</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>岩田　知機（イワタ　チキ）</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" s="1"/>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
           <t>2026/06/11 12:06</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>岩田　知機（イワタ　チキ）</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>https://yububuyvyu.github.io/map/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/PR3NWxo7woyLZb0O</t>
         </is>
       </c>
-      <c r="J3" s="1"/>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M3" s="1"/>
-      <c r="N3" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O3" s="1"/>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="J4" s="1"/>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O4" s="1"/>
+      <c r="P4" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="Q4" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="R4" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="S4" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T3" s="4" t="inlineStr">
+      <c r="T4" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U3" s="4" t="inlineStr">
+      <c r="U4" s="4" t="inlineStr">
         <is>
           <t>10.30.60.225</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>1254510435</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>岡野　俊介（オカノ　シュンスケ）</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>2026/06/11 10:06</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr">
         <is>
           <t>岡野　俊介（オカノ　シュンスケ）</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/94PGWnoK52qoaLRV
 https://osyunsuke.github.io/map-01/
 https://github.com/OSyunsuke/map-01</t>
         </is>
       </c>
-      <c r="J4" s="1"/>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M4" s="1"/>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O4" s="1"/>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="J5" s="1"/>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5" s="1"/>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" s="1"/>
+      <c r="P5" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q4" s="4" t="inlineStr">
+      <c r="Q5" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R4" s="4" t="inlineStr">
+      <c r="R5" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S4" s="4" t="inlineStr">
+      <c r="S5" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T4" s="4" t="inlineStr">
+      <c r="T5" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U4" s="4" t="inlineStr">
+      <c r="U5" s="4" t="inlineStr">
         <is>
           <t>10.30.59.79</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>1254510625</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>日下　智弥（クサカ　トモヤ）</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F5" s="1"/>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" s="1"/>
+      <c r="G6" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 23:15</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>日下　智弥（クサカ　トモヤ）</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>https://a250343t-alt.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/94PGWnoq7ML4aLRV</t>
         </is>
       </c>
-      <c r="J5" s="1"/>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M5" s="1"/>
-      <c r="N5" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O5" s="1"/>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="J6" s="1"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="1"/>
+      <c r="P6" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q5" s="4" t="inlineStr">
+      <c r="Q6" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R5" s="4" t="inlineStr">
+      <c r="R6" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S5" s="4" t="inlineStr">
+      <c r="S6" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T5" s="4" t="inlineStr">
+      <c r="T6" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U5" s="4" t="inlineStr">
+      <c r="U6" s="4" t="inlineStr">
         <is>
           <t>106.73.185.199</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>1254510865</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>佐藤　太陽（サトウ　タイヨウ）</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F6" s="1"/>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:12</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>佐藤　太陽（サトウ　タイヨウ）</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/BJkrQA9XKek4QEge
 https://satotaiyo0503.github.io/map02/
 https://github.com/SatoTaiyo0503/map02</t>
         </is>
       </c>
-      <c r="J6" s="1"/>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M6" s="1"/>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O6" s="1"/>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="J7" s="1"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="1"/>
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="T7" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>153.232.156.182</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>1254511136</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>滝澤　恵豪（タキザワ　ケイゴ）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 21:18</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>滝澤　恵豪（タキザワ　ケイゴ）</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/YBl3Z2O3Ge47Wv16
 https://keigotakky3-eng.github.io/map01/</t>
         </is>
       </c>
-      <c r="J7" s="1"/>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M7" s="1"/>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O7" s="1"/>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="J8" s="1"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" s="1"/>
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S7" s="4" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>222.6.232.21</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>1254511251</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>土屋　響輝（ツチヤ　ヒビキ）</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:22</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>土屋　響輝（ツチヤ　ヒビキ）</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Padlet URL
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/lkROZPpJDzrMZjMg
@@ -833,194 +925,103 @@
 https://github.com/hibiki20060716/map01.git</t>
         </is>
       </c>
-      <c r="J8" s="1"/>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M8" s="1"/>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O8" s="1"/>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="J9" s="1"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" s="1"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" s="1"/>
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr">
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="T9" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr">
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>61.23.189.153</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>1254511912</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>金澤　一華（カナザワ　イチカ）</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 22:04</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>金澤　一華（カナザワ　イチカ）</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>https://a250989i-code.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/e9YpQNpzDj2lWxjM</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>元々南柏での空きコマを潰せる場所マップを作ろうと思っていましたが、今回の講義でみんなのサイトを見たときに音楽をつけたり、飛べるようにしたりできる面白いものを作りたいと思ってプロジェクトの内容を変えてしまいました。まだ私が自信を持って見せれるものではないので、サイトを開いたらもっと心躍るものを作りたいです。</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M9" s="1"/>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O9" s="1"/>
-      <c r="P9" s="4" t="inlineStr">
-        <is>
-          <t>2年</t>
-        </is>
-      </c>
-      <c r="Q9" s="4" t="inlineStr">
-        <is>
-          <t>3セメスタ</t>
-        </is>
-      </c>
-      <c r="R9" s="4" t="inlineStr">
-        <is>
-          <t>麗澤大学 経済学部 経済学科 経済</t>
-        </is>
-      </c>
-      <c r="S9" s="4" t="inlineStr">
-        <is>
-          <t>2025年度 春</t>
-        </is>
-      </c>
-      <c r="T9" s="4" t="inlineStr">
-        <is>
-          <t>進級</t>
-        </is>
-      </c>
-      <c r="U9" s="4" t="inlineStr">
-        <is>
-          <t>118.156.108.198</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>1254512085</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>宮城　大空（ミヤギ　ソラ）</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>2026/06/16 09:52</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t>宮城　大空（ミヤギ　ソラ）</t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/7p6nvbdgst-dev/map01.githttps://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/zV61Q6xkVYLbWO98</t>
-        </is>
-      </c>
-      <c r="J10" s="1"/>
       <c r="K10" s="4" t="inlineStr">
         <is>
           <t/>
@@ -1065,19 +1066,19 @@
       </c>
       <c r="U10" s="4" t="inlineStr">
         <is>
-          <t>153.169.20.190</t>
+          <t>118.156.108.198</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>1254690352</t>
+          <t>1254512085</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+          <t>宮城　大空（ミヤギ　ソラ）</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -1098,199 +1099,290 @@
       <c r="F11" s="1"/>
       <c r="G11" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 09:52</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>宮城　大空（ミヤギ　ソラ）</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/7p6nvbdgst-dev/map01.githttps://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/zV61Q6xkVYLbWO98</t>
+        </is>
+      </c>
+      <c r="J11" s="1"/>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O11" s="1"/>
+      <c r="P11" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q11" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R11" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 経済学部 経済学科 経済</t>
+        </is>
+      </c>
+      <c r="S11" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T11" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U11" s="4" t="inlineStr">
+        <is>
+          <t>153.169.20.190</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>1254690352</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F12" s="1"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
           <t>2026/06/11 11:20</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2NvBGBZgP7
 https://jyb1472.github.io/map01/</t>
         </is>
       </c>
-      <c r="J11" s="1"/>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M11" s="1"/>
-      <c r="N11" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O11" s="1"/>
-      <c r="P11" s="4" t="inlineStr">
+      <c r="J12" s="1"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O12" s="1"/>
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q11" s="4" t="inlineStr">
+      <c r="Q12" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R11" s="4" t="inlineStr">
+      <c r="R12" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際交流国際協力</t>
         </is>
       </c>
-      <c r="S11" s="4" t="inlineStr">
+      <c r="S12" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T11" s="4" t="inlineStr">
+      <c r="T12" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U11" s="4" t="inlineStr">
+      <c r="U12" s="4" t="inlineStr">
         <is>
           <t>10.30.50.131</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>1254690435</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F12" s="1"/>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 19:26</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿のURL: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/j40PQDYqXVweZvXB
 GitHub Pages のURL : https://nejihyugamsp.github.io/UNESCO-World-Map/</t>
         </is>
       </c>
-      <c r="J12" s="1"/>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M12" s="1"/>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O12" s="1"/>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="J13" s="1"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O13" s="1"/>
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R12" s="4" t="inlineStr">
+      <c r="R13" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際社会</t>
         </is>
       </c>
-      <c r="S12" s="4" t="inlineStr">
+      <c r="S13" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T12" s="4" t="inlineStr">
+      <c r="T13" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U12" s="4" t="inlineStr">
+      <c r="U13" s="4" t="inlineStr">
         <is>
           <t>126.114.113.205</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>1254810059</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F13" s="1"/>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:02</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2jDgRMZgP7
@@ -1298,1114 +1390,1023 @@
 https://awano-kakeru.github.io/map01/</t>
         </is>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O13" s="1"/>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="J14" s="1"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" s="1"/>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr">
+      <c r="S14" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
+      <c r="T14" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
+      <c r="U14" s="4" t="inlineStr">
         <is>
           <t>10.30.25.13</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>1254810075</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F14" s="1"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 22:17</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Padlet:https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/e9YpQNpzDoXDWxjM
 GitHub Pages:https://a250818h-ai.github.io/map01/</t>
         </is>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O14" s="1"/>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="J15" s="1"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" s="1"/>
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="T15" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr">
+      <c r="U15" s="4" t="inlineStr">
         <is>
           <t>106.160.0.32</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>1254810124</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 23:49</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>https://ayuma-wp.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/x5A7aroMvBBxQwr6</t>
         </is>
       </c>
-      <c r="J15" s="1"/>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O15" s="1"/>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="J16" s="1"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr">
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R15" s="4" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr">
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
+      <c r="T16" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr">
+      <c r="U16" s="4" t="inlineStr">
         <is>
           <t>36.12.197.93</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>1254810140</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 06:47</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjAKwnqa0OX
 https://kazu2856.github.io/fammap/
 https://github.com/kazu2856/fammap</t>
         </is>
       </c>
-      <c r="J16" s="1"/>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M16" s="1"/>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O16" s="1"/>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="J17" s="1"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" s="1"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O17" s="1"/>
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="Q17" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R16" s="4" t="inlineStr">
+      <c r="R17" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
+      <c r="T17" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr">
+      <c r="U17" s="4" t="inlineStr">
         <is>
           <t>133.114.4.189</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>1254810166</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:57</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Padlet: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/R7dXadN53qbeZ6bl
 git hub: a250827o-blip.github.io/map02/</t>
         </is>
       </c>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O17" s="1"/>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="J18" s="1"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" s="1"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" s="1"/>
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R17" s="4" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr">
+      <c r="U18" s="4" t="inlineStr">
         <is>
           <t>153.241.128.1</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>1254810174</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:50</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/do3MQJwe0LnOZ15w
 https://shun-onitsuka.github.io/map01/</t>
         </is>
       </c>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M18" s="1"/>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O18" s="1"/>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="J19" s="1"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M19" s="1"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O19" s="1"/>
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
+      <c r="Q19" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R18" s="4" t="inlineStr">
+      <c r="R19" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
+      <c r="S19" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T18" s="4" t="inlineStr">
+      <c r="T19" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
+      <c r="U19" s="4" t="inlineStr">
         <is>
           <t>59.132.16.22</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>1254810182</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>2026/06/09 16:14</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/J24jalobBy6YW0A1
 https://github.com/a250829s-code/earth-map.git
 https://a250829s-code.github.io/earth-map/</t>
         </is>
       </c>
-      <c r="J19" s="1"/>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M19" s="1"/>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O19" s="1"/>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="J20" s="1"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M20" s="1"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O20" s="1"/>
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q19" s="4" t="inlineStr">
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R19" s="4" t="inlineStr">
+      <c r="R20" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
+      <c r="S20" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
+      <c r="T20" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
+      <c r="U20" s="4" t="inlineStr">
         <is>
           <t>10.30.60.247</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>1254810299</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 13:32</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/AL83Wz7JPBnXa0Pg(padlet)
 https://1254810299.github.io/map01/(gitpages)</t>
         </is>
       </c>
-      <c r="J20" s="1"/>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M20" s="1"/>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O20" s="1"/>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="J21" s="1"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O21" s="1"/>
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
+      <c r="Q21" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R20" s="4" t="inlineStr">
+      <c r="R21" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
+      <c r="S21" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
+      <c r="U21" s="4" t="inlineStr">
         <is>
           <t>10.30.25.6</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>1254810372</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 12:36</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/XGyBQb1x2VmgaL6K 
 https://sari6641.github.io/map01/</t>
         </is>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" s="1"/>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" s="1"/>
-      <c r="P21" s="4" t="inlineStr">
+      <c r="J22" s="1"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M22" s="1"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O22" s="1"/>
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="inlineStr">
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R21" s="4" t="inlineStr">
+      <c r="R22" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
+      <c r="S22" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
+      <c r="T22" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr">
+      <c r="U22" s="4" t="inlineStr">
         <is>
           <t>106.128.107.23</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>1254810405</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F23" s="1"/>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:52</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Xb8YaLpw5XlJayn1
 https://sibaba615.github.io/map1/
 https://github.com/sibaba615/map1</t>
         </is>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" s="1"/>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" s="1"/>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="J23" s="1"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" s="1"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O23" s="1"/>
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="Q23" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R22" s="4" t="inlineStr">
+      <c r="R23" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
+      <c r="S23" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
+      <c r="T23" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
+      <c r="U23" s="4" t="inlineStr">
         <is>
           <t>219.104.130.164</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>1254810413</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" s="1"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:07</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/yEPVZkoXldopZb0Y
 https://joe-0711.github.io/map01/
 https://github.com/joe-0711/map01</t>
         </is>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" s="1"/>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" s="1"/>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="J24" s="1"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" s="1"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O24" s="1"/>
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="inlineStr">
+      <c r="Q24" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="R24" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S24" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
+      <c r="T24" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
+      <c r="U24" s="4" t="inlineStr">
         <is>
           <t>60.93.159.60</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>1254810512</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:11</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>https://taketaago.github.io/map01/
 https://github.com/taketaago/map01
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/L8KjW9vyykk2aJbv</t>
         </is>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" s="1"/>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" s="1"/>
-      <c r="P24" s="4" t="inlineStr">
-        <is>
-          <t>2年</t>
-        </is>
-      </c>
-      <c r="Q24" s="4" t="inlineStr">
-        <is>
-          <t>3セメスタ</t>
-        </is>
-      </c>
-      <c r="R24" s="4" t="inlineStr">
-        <is>
-          <t>麗澤大学 工学部 工学科 情報システム工学</t>
-        </is>
-      </c>
-      <c r="S24" s="4" t="inlineStr">
-        <is>
-          <t>2025年度 春</t>
-        </is>
-      </c>
-      <c r="T24" s="4" t="inlineStr">
-        <is>
-          <t>進級</t>
-        </is>
-      </c>
-      <c r="U24" s="4" t="inlineStr">
-        <is>
-          <t>150.91.180.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>1254810562</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>2026/06/10 19:53</t>
-        </is>
-      </c>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
-        </is>
-      </c>
       <c r="J25" s="1"/>
       <c r="K25" s="4" t="inlineStr">
         <is>
@@ -2451,19 +2452,19 @@
       </c>
       <c r="U25" s="4" t="inlineStr">
         <is>
-          <t>1.115.90.218</t>
+          <t>150.91.180.64</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>1254810588</t>
+          <t>1254810562</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>野村　隆介（ノムラ　リュウスケ）</t>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2484,617 +2485,708 @@
       <c r="F26" s="1"/>
       <c r="G26" s="5" t="inlineStr">
         <is>
+          <t>2026/06/10 19:53</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
+        </is>
+      </c>
+      <c r="J26" s="1"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M26" s="1"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O26" s="1"/>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q26" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R26" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 工学部 工学科 情報システム工学</t>
+        </is>
+      </c>
+      <c r="S26" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T26" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U26" s="4" t="inlineStr">
+        <is>
+          <t>1.115.90.218</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>1254810588</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>野村　隆介（ノムラ　リュウスケ）</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
           <t>2026/06/13 13:52</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>野村　隆介（ノムラ　リュウスケ）</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mDRxWBq0x4rOZjb1
 https://nomuraryuusuke.github.io/map----/</t>
         </is>
       </c>
-      <c r="J26" s="1"/>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M26" s="1"/>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O26" s="1"/>
-      <c r="P26" s="4" t="inlineStr">
+      <c r="J27" s="1"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M27" s="1"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O27" s="1"/>
+      <c r="P27" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q26" s="4" t="inlineStr">
+      <c r="Q27" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R26" s="4" t="inlineStr">
+      <c r="R27" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S26" s="4" t="inlineStr">
+      <c r="S27" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T26" s="4" t="inlineStr">
+      <c r="T27" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U26" s="4" t="inlineStr">
+      <c r="U27" s="4" t="inlineStr">
         <is>
           <t>118.241.60.18</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
         <is>
           <t>1254810736</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F28" s="1"/>
+      <c r="G28" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 13:34</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/jpoxajk68LqOQbPE
 https://yuu08080.github.io/map01/</t>
         </is>
       </c>
-      <c r="J27" s="1"/>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M27" s="1"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O27" s="1"/>
-      <c r="P27" s="4" t="inlineStr">
+      <c r="J28" s="1"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M28" s="1"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q27" s="4" t="inlineStr">
+      <c r="Q28" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R27" s="4" t="inlineStr">
+      <c r="R28" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S27" s="4" t="inlineStr">
+      <c r="S28" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
+      <c r="T28" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
+      <c r="U28" s="4" t="inlineStr">
         <is>
           <t>10.30.59.77</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>1254810801</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F29" s="1"/>
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:23</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjABEY3a0OX
  https://souta-1213.github.io/map01/</t>
         </is>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M28" s="1"/>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O28" s="1"/>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="J29" s="1"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M29" s="1"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O29" s="1"/>
+      <c r="P29" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
+      <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R28" s="4" t="inlineStr">
+      <c r="R29" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S28" s="4" t="inlineStr">
+      <c r="S29" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
+      <c r="T29" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U28" s="4" t="inlineStr">
+      <c r="U29" s="4" t="inlineStr">
         <is>
           <t>126.249.152.193</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>1254810827</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F30" s="1"/>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:14</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/LNV1Q7y77JrrWmq3
 https://yaegashi0314.github.io/map001/</t>
         </is>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M29" s="1"/>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O29" s="1"/>
-      <c r="P29" s="4" t="inlineStr">
+      <c r="J30" s="1"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M30" s="1"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O30" s="1"/>
+      <c r="P30" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R29" s="4" t="inlineStr">
+      <c r="R30" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr">
+      <c r="S30" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
+      <c r="T30" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr">
+      <c r="U30" s="4" t="inlineStr">
         <is>
           <t>118.83.190.225</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>1254810926</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" s="1"/>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:55</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mlNDZ3OGGDrqZznG
 https://github.com/a250903y-gif/a250903y-gif.github.io.git</t>
         </is>
       </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M30" s="1"/>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O30" s="1"/>
-      <c r="P30" s="4" t="inlineStr">
+      <c r="J31" s="1"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M31" s="1"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O31" s="1"/>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
+      <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R30" s="4" t="inlineStr">
+      <c r="R31" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S30" s="4" t="inlineStr">
+      <c r="S31" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
+      <c r="T31" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr">
+      <c r="U31" s="4" t="inlineStr">
         <is>
           <t>116.82.97.244</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>1254810992</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F32" s="1"/>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:01</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Ae2Ravoe2PpOQnz4
 https://github.com/edwin379/train
 https://train-5dwy.onrender.com/</t>
         </is>
       </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M31" s="1"/>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O31" s="1"/>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="J32" s="1"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M32" s="1"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O32" s="1"/>
+      <c r="P32" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q32" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R31" s="4" t="inlineStr">
+      <c r="R32" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr">
+      <c r="S32" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
+      <c r="T32" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U31" s="4" t="inlineStr">
+      <c r="U32" s="4" t="inlineStr">
         <is>
           <t>10.30.56.85</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>1254820222</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 20:09</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/4b3zaMpVDXA9W2j7
 https://github.com/a250927s-create/HIPHOPMAP.git</t>
         </is>
       </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M32" s="1"/>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O32" s="1"/>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="J33" s="1"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M33" s="1"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O33" s="1"/>
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q33" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr">
+      <c r="R33" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 ロボティクス</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr">
+      <c r="S33" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
+      <c r="T33" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
+      <c r="U33" s="4" t="inlineStr">
         <is>
           <t>10.30.48.85</t>
         </is>

</xml_diff>

<commit_message>
in class midterm updates
</commit_message>
<xml_diff>
--- a/kadai/week08/midterms.xlsx
+++ b/kadai/week08/midterms.xlsx
@@ -3010,12 +3010,12 @@
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>1254810992</t>
+          <t>1254810976</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
+          <t>坂本　快（サカモト　カイ）</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3036,157 +3036,249 @@
       <c r="F32" s="1"/>
       <c r="G32" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 10:39</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>坂本　快（サカモト　カイ）</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>https://kai-sakamoto.github.io/map01/
+https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/dMA1W85Rz97Xa4OV</t>
+        </is>
+      </c>
+      <c r="J32" s="1"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M32" s="1"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O32" s="1"/>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 工学部 工学科 情報システム工学</t>
+        </is>
+      </c>
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U32" s="4" t="inlineStr">
+        <is>
+          <t>10.30.25.100</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>1254810992</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
           <t>2026/06/12 14:01</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Ae2Ravoe2PpOQnz4
 https://github.com/edwin379/train
 https://train-5dwy.onrender.com/</t>
         </is>
       </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M32" s="1"/>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O32" s="1"/>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="J33" s="1"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M33" s="1"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O33" s="1"/>
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q33" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr">
+      <c r="R33" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr">
+      <c r="S33" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
+      <c r="T33" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
+      <c r="U33" s="4" t="inlineStr">
         <is>
           <t>10.30.56.85</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>1254820222</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 20:09</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/4b3zaMpVDXA9W2j7
 https://github.com/a250927s-create/HIPHOPMAP.git</t>
         </is>
       </c>
-      <c r="J33" s="1"/>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M33" s="1"/>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O33" s="1"/>
-      <c r="P33" s="4" t="inlineStr">
+      <c r="J34" s="1"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M34" s="1"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O34" s="1"/>
+      <c r="P34" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
+      <c r="Q34" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R33" s="4" t="inlineStr">
+      <c r="R34" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 ロボティクス</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr">
+      <c r="S34" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
+      <c r="T34" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
+      <c r="U34" s="4" t="inlineStr">
         <is>
           <t>10.30.48.85</t>
         </is>

</xml_diff>

<commit_message>
in class final update for midterms
</commit_message>
<xml_diff>
--- a/kadai/week08/midterms.xlsx
+++ b/kadai/week08/midterms.xlsx
@@ -1164,12 +1164,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>1254690352</t>
+          <t>1254512134</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+          <t>荒井　聡（アライ　アキラ）</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1190,199 +1190,290 @@
       <c r="F12" s="1"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 10:57</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>荒井　聡（アライ　アキラ）</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>https://gis-araiakira.github.io/map01/</t>
+        </is>
+      </c>
+      <c r="J12" s="1"/>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O12" s="1"/>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R12" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 経済学部 経済学科 経済</t>
+        </is>
+      </c>
+      <c r="S12" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T12" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U12" s="4" t="inlineStr">
+        <is>
+          <t>10.30.57.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>1254690352</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F13" s="1"/>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
           <t>2026/06/11 11:20</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H13" s="4" t="inlineStr">
         <is>
           <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I13" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2NvBGBZgP7
 https://jyb1472.github.io/map01/</t>
         </is>
       </c>
-      <c r="J12" s="1"/>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M12" s="1"/>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O12" s="1"/>
-      <c r="P12" s="4" t="inlineStr">
+      <c r="J13" s="1"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O13" s="1"/>
+      <c r="P13" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q12" s="4" t="inlineStr">
+      <c r="Q13" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R12" s="4" t="inlineStr">
+      <c r="R13" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際交流国際協力</t>
         </is>
       </c>
-      <c r="S12" s="4" t="inlineStr">
+      <c r="S13" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T12" s="4" t="inlineStr">
+      <c r="T13" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U12" s="4" t="inlineStr">
+      <c r="U13" s="4" t="inlineStr">
         <is>
           <t>10.30.50.131</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>1254690435</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C14" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F13" s="1"/>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 19:26</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿のURL: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/j40PQDYqXVweZvXB
 GitHub Pages のURL : https://nejihyugamsp.github.io/UNESCO-World-Map/</t>
         </is>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O13" s="1"/>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="J14" s="1"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" s="1"/>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際社会</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr">
+      <c r="S14" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
+      <c r="T14" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
+      <c r="U14" s="4" t="inlineStr">
         <is>
           <t>126.114.113.205</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>1254810059</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F14" s="1"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:02</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2jDgRMZgP7
@@ -1390,1114 +1481,1023 @@
 https://awano-kakeru.github.io/map01/</t>
         </is>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O14" s="1"/>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="J15" s="1"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" s="1"/>
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="T15" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr">
+      <c r="U15" s="4" t="inlineStr">
         <is>
           <t>10.30.25.13</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>1254810075</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 22:17</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Padlet:https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/e9YpQNpzDoXDWxjM
 GitHub Pages:https://a250818h-ai.github.io/map01/</t>
         </is>
       </c>
-      <c r="J15" s="1"/>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O15" s="1"/>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="J16" s="1"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr">
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R15" s="4" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr">
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
+      <c r="T16" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr">
+      <c r="U16" s="4" t="inlineStr">
         <is>
           <t>106.160.0.32</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>1254810124</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 23:49</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>https://ayuma-wp.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/x5A7aroMvBBxQwr6</t>
         </is>
       </c>
-      <c r="J16" s="1"/>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M16" s="1"/>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O16" s="1"/>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="J17" s="1"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" s="1"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O17" s="1"/>
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="Q17" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R16" s="4" t="inlineStr">
+      <c r="R17" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
+      <c r="T17" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr">
+      <c r="U17" s="4" t="inlineStr">
         <is>
           <t>36.12.197.93</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>1254810140</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 06:47</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjAKwnqa0OX
 https://kazu2856.github.io/fammap/
 https://github.com/kazu2856/fammap</t>
         </is>
       </c>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O17" s="1"/>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="J18" s="1"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" s="1"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" s="1"/>
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R17" s="4" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr">
+      <c r="U18" s="4" t="inlineStr">
         <is>
           <t>133.114.4.189</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>1254810166</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:57</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Padlet: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/R7dXadN53qbeZ6bl
 git hub: a250827o-blip.github.io/map02/</t>
         </is>
       </c>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M18" s="1"/>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O18" s="1"/>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="J19" s="1"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M19" s="1"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O19" s="1"/>
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
+      <c r="Q19" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R18" s="4" t="inlineStr">
+      <c r="R19" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
+      <c r="S19" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T18" s="4" t="inlineStr">
+      <c r="T19" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
+      <c r="U19" s="4" t="inlineStr">
         <is>
           <t>153.241.128.1</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>1254810174</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:50</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/do3MQJwe0LnOZ15w
 https://shun-onitsuka.github.io/map01/</t>
         </is>
       </c>
-      <c r="J19" s="1"/>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M19" s="1"/>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O19" s="1"/>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="J20" s="1"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M20" s="1"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O20" s="1"/>
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q19" s="4" t="inlineStr">
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R19" s="4" t="inlineStr">
+      <c r="R20" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
+      <c r="S20" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
+      <c r="T20" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
+      <c r="U20" s="4" t="inlineStr">
         <is>
           <t>59.132.16.22</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>1254810182</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>2026/06/09 16:14</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/J24jalobBy6YW0A1
 https://github.com/a250829s-code/earth-map.git
 https://a250829s-code.github.io/earth-map/</t>
         </is>
       </c>
-      <c r="J20" s="1"/>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M20" s="1"/>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O20" s="1"/>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="J21" s="1"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O21" s="1"/>
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
+      <c r="Q21" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R20" s="4" t="inlineStr">
+      <c r="R21" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
+      <c r="S21" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
+      <c r="U21" s="4" t="inlineStr">
         <is>
           <t>10.30.60.247</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>1254810299</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 13:32</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/AL83Wz7JPBnXa0Pg(padlet)
 https://1254810299.github.io/map01/(gitpages)</t>
         </is>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" s="1"/>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" s="1"/>
-      <c r="P21" s="4" t="inlineStr">
+      <c r="J22" s="1"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M22" s="1"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O22" s="1"/>
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="inlineStr">
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R21" s="4" t="inlineStr">
+      <c r="R22" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
+      <c r="S22" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
+      <c r="T22" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr">
+      <c r="U22" s="4" t="inlineStr">
         <is>
           <t>10.30.25.6</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>1254810372</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F23" s="1"/>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 12:36</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/XGyBQb1x2VmgaL6K 
 https://sari6641.github.io/map01/</t>
         </is>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" s="1"/>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" s="1"/>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="J23" s="1"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" s="1"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O23" s="1"/>
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="Q23" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R22" s="4" t="inlineStr">
+      <c r="R23" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
+      <c r="S23" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
+      <c r="T23" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
+      <c r="U23" s="4" t="inlineStr">
         <is>
           <t>106.128.107.23</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>1254810405</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" s="1"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:52</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Xb8YaLpw5XlJayn1
 https://sibaba615.github.io/map1/
 https://github.com/sibaba615/map1</t>
         </is>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" s="1"/>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" s="1"/>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="J24" s="1"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" s="1"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O24" s="1"/>
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="inlineStr">
+      <c r="Q24" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="R24" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S24" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
+      <c r="T24" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
+      <c r="U24" s="4" t="inlineStr">
         <is>
           <t>219.104.130.164</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>1254810413</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:07</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/yEPVZkoXldopZb0Y
 https://joe-0711.github.io/map01/
 https://github.com/joe-0711/map01</t>
         </is>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" s="1"/>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" s="1"/>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="J25" s="1"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M25" s="1"/>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O25" s="1"/>
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
+      <c r="Q25" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R24" s="4" t="inlineStr">
+      <c r="R25" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr">
+      <c r="S25" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="T25" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
+      <c r="U25" s="4" t="inlineStr">
         <is>
           <t>60.93.159.60</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>1254810512</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F26" s="1"/>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:11</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>https://taketaago.github.io/map01/
 https://github.com/taketaago/map01
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/L8KjW9vyykk2aJbv</t>
         </is>
       </c>
-      <c r="J25" s="1"/>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M25" s="1"/>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" s="1"/>
-      <c r="P25" s="4" t="inlineStr">
-        <is>
-          <t>2年</t>
-        </is>
-      </c>
-      <c r="Q25" s="4" t="inlineStr">
-        <is>
-          <t>3セメスタ</t>
-        </is>
-      </c>
-      <c r="R25" s="4" t="inlineStr">
-        <is>
-          <t>麗澤大学 工学部 工学科 情報システム工学</t>
-        </is>
-      </c>
-      <c r="S25" s="4" t="inlineStr">
-        <is>
-          <t>2025年度 春</t>
-        </is>
-      </c>
-      <c r="T25" s="4" t="inlineStr">
-        <is>
-          <t>進級</t>
-        </is>
-      </c>
-      <c r="U25" s="4" t="inlineStr">
-        <is>
-          <t>150.91.180.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>1254810562</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>2026/06/10 19:53</t>
-        </is>
-      </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
-        </is>
-      </c>
       <c r="J26" s="1"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
@@ -2543,19 +2543,19 @@
       </c>
       <c r="U26" s="4" t="inlineStr">
         <is>
-          <t>1.115.90.218</t>
+          <t>150.91.180.64</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>1254810588</t>
+          <t>1254810562</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>野村　隆介（ノムラ　リュウスケ）</t>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2576,709 +2576,892 @@
       <c r="F27" s="1"/>
       <c r="G27" s="5" t="inlineStr">
         <is>
+          <t>2026/06/10 19:53</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
+        </is>
+      </c>
+      <c r="J27" s="1"/>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M27" s="1"/>
+      <c r="N27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O27" s="1"/>
+      <c r="P27" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q27" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R27" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 工学部 工学科 情報システム工学</t>
+        </is>
+      </c>
+      <c r="S27" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T27" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U27" s="4" t="inlineStr">
+        <is>
+          <t>1.115.90.218</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>1254810588</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>野村　隆介（ノムラ　リュウスケ）</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F28" s="1"/>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
           <t>2026/06/13 13:52</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>野村　隆介（ノムラ　リュウスケ）</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mDRxWBq0x4rOZjb1
 https://nomuraryuusuke.github.io/map----/</t>
         </is>
       </c>
-      <c r="J27" s="1"/>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M27" s="1"/>
-      <c r="N27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O27" s="1"/>
-      <c r="P27" s="4" t="inlineStr">
+      <c r="J28" s="1"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M28" s="1"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q27" s="4" t="inlineStr">
+      <c r="Q28" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R27" s="4" t="inlineStr">
+      <c r="R28" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S27" s="4" t="inlineStr">
+      <c r="S28" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T27" s="4" t="inlineStr">
+      <c r="T28" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U27" s="4" t="inlineStr">
+      <c r="U28" s="4" t="inlineStr">
         <is>
           <t>118.241.60.18</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
         <is>
           <t>1254810736</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B29" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F28" s="1"/>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F29" s="1"/>
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 13:34</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/jpoxajk68LqOQbPE
 https://yuu08080.github.io/map01/</t>
         </is>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M28" s="1"/>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O28" s="1"/>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="J29" s="1"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M29" s="1"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O29" s="1"/>
+      <c r="P29" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
+      <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R28" s="4" t="inlineStr">
+      <c r="R29" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S28" s="4" t="inlineStr">
+      <c r="S29" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
+      <c r="T29" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U28" s="4" t="inlineStr">
+      <c r="U29" s="4" t="inlineStr">
         <is>
           <t>10.30.59.77</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>1254810794</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>桃井　優（モモイ　ユウ）</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F30" s="1"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>2026/06/16 10:59</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>桃井　優（モモイ　ユウ）</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/j40PQDYDoE3XZvXB
+https://a250890y-cmd.github.io/memory_map_web/</t>
+        </is>
+      </c>
+      <c r="J30" s="1"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M30" s="1"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O30" s="1"/>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q30" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R30" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 工学部 工学科 情報システム工学</t>
+        </is>
+      </c>
+      <c r="S30" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T30" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U30" s="4" t="inlineStr">
+        <is>
+          <t>10.30.56.176</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>1254810801</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:23</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjABEY3a0OX
  https://souta-1213.github.io/map01/</t>
         </is>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M29" s="1"/>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O29" s="1"/>
-      <c r="P29" s="4" t="inlineStr">
+      <c r="J31" s="1"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M31" s="1"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O31" s="1"/>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R29" s="4" t="inlineStr">
+      <c r="R31" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr">
+      <c r="S31" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
+      <c r="T31" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr">
+      <c r="U31" s="4" t="inlineStr">
         <is>
           <t>126.249.152.193</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>1254810827</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" s="1"/>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F32" s="1"/>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:14</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/LNV1Q7y77JrrWmq3
 https://yaegashi0314.github.io/map001/</t>
         </is>
       </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M30" s="1"/>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O30" s="1"/>
-      <c r="P30" s="4" t="inlineStr">
+      <c r="J32" s="1"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M32" s="1"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O32" s="1"/>
+      <c r="P32" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
+      <c r="Q32" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R30" s="4" t="inlineStr">
+      <c r="R32" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S30" s="4" t="inlineStr">
+      <c r="S32" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
+      <c r="T32" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr">
+      <c r="U32" s="4" t="inlineStr">
         <is>
           <t>118.83.190.225</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>1254810926</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:55</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mlNDZ3OGGDrqZznG
 https://github.com/a250903y-gif/a250903y-gif.github.io.git</t>
         </is>
       </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M31" s="1"/>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O31" s="1"/>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="J33" s="1"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M33" s="1"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O33" s="1"/>
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q33" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R31" s="4" t="inlineStr">
+      <c r="R33" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr">
+      <c r="S33" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
+      <c r="T33" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U31" s="4" t="inlineStr">
+      <c r="U33" s="4" t="inlineStr">
         <is>
           <t>116.82.97.244</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>1254810976</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>坂本　快（サカモト　カイ）</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 10:39</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>坂本　快（サカモト　カイ）</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>https://kai-sakamoto.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/dMA1W85Rz97Xa4OV</t>
         </is>
       </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M32" s="1"/>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O32" s="1"/>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="J34" s="1"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M34" s="1"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O34" s="1"/>
+      <c r="P34" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q34" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr">
+      <c r="R34" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr">
+      <c r="S34" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
+      <c r="T34" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
+      <c r="U34" s="4" t="inlineStr">
         <is>
           <t>10.30.25.100</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>1254810992</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:01</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Ae2Ravoe2PpOQnz4
 https://github.com/edwin379/train
 https://train-5dwy.onrender.com/</t>
         </is>
       </c>
-      <c r="J33" s="1"/>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M33" s="1"/>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O33" s="1"/>
-      <c r="P33" s="4" t="inlineStr">
+      <c r="J35" s="1"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M35" s="1"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O35" s="1"/>
+      <c r="P35" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
+      <c r="Q35" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R33" s="4" t="inlineStr">
+      <c r="R35" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr">
+      <c r="S35" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
+      <c r="T35" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
+      <c r="U35" s="4" t="inlineStr">
         <is>
           <t>10.30.56.85</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>1254820222</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F34" s="1"/>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 20:09</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/4b3zaMpVDXA9W2j7
 https://github.com/a250927s-create/HIPHOPMAP.git</t>
         </is>
       </c>
-      <c r="J34" s="1"/>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M34" s="1"/>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O34" s="1"/>
-      <c r="P34" s="4" t="inlineStr">
+      <c r="J36" s="1"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M36" s="1"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O36" s="1"/>
+      <c r="P36" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q34" s="4" t="inlineStr">
+      <c r="Q36" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R34" s="4" t="inlineStr">
+      <c r="R36" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 ロボティクス</t>
         </is>
       </c>
-      <c r="S34" s="4" t="inlineStr">
+      <c r="S36" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T34" s="4" t="inlineStr">
+      <c r="T36" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U34" s="4" t="inlineStr">
+      <c r="U36" s="4" t="inlineStr">
         <is>
           <t>10.30.48.85</t>
         </is>

</xml_diff>

<commit_message>
midterm updates after class
</commit_message>
<xml_diff>
--- a/kadai/week08/midterms.xlsx
+++ b/kadai/week08/midterms.xlsx
@@ -606,12 +606,12 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>1254510625</t>
+          <t>1254510534</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>日下　智弥（クサカ　トモヤ）</t>
+          <t>川合　悠（カワイ　ユウ）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -632,292 +632,384 @@
       <c r="F6" s="1"/>
       <c r="G6" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 11:30</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>川合　悠（カワイ　ユウ）</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/goElQyOoEVDmW3yY
+https://a250334y-create.github.io/map01/</t>
+        </is>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M6" s="1"/>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O6" s="1"/>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R6" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 経済学部 経済学科 経済</t>
+        </is>
+      </c>
+      <c r="S6" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T6" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U6" s="4" t="inlineStr">
+        <is>
+          <t>10.30.57.104</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>1254510625</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>日下　智弥（クサカ　トモヤ）</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" s="1"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
           <t>2026/06/15 23:15</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>日下　智弥（クサカ　トモヤ）</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t>https://a250343t-alt.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/94PGWnoq7ML4aLRV</t>
         </is>
       </c>
-      <c r="J6" s="1"/>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M6" s="1"/>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O6" s="1"/>
-      <c r="P6" s="4" t="inlineStr">
+      <c r="J7" s="1"/>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M7" s="1"/>
+      <c r="N7" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O7" s="1"/>
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q6" s="4" t="inlineStr">
+      <c r="Q7" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R6" s="4" t="inlineStr">
+      <c r="R7" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S6" s="4" t="inlineStr">
+      <c r="S7" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T6" s="4" t="inlineStr">
+      <c r="T7" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U6" s="4" t="inlineStr">
+      <c r="U7" s="4" t="inlineStr">
         <is>
           <t>106.73.185.199</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>1254510865</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>佐藤　太陽（サトウ　タイヨウ）</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" s="1"/>
+      <c r="G8" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:12</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>佐藤　太陽（サトウ　タイヨウ）</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I8" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/BJkrQA9XKek4QEge
 https://satotaiyo0503.github.io/map02/
 https://github.com/SatoTaiyo0503/map02</t>
         </is>
       </c>
-      <c r="J7" s="1"/>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M7" s="1"/>
-      <c r="N7" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O7" s="1"/>
-      <c r="P7" s="4" t="inlineStr">
+      <c r="J8" s="1"/>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M8" s="1"/>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O8" s="1"/>
+      <c r="P8" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q7" s="4" t="inlineStr">
+      <c r="Q8" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R7" s="4" t="inlineStr">
+      <c r="R8" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S7" s="4" t="inlineStr">
+      <c r="S8" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T7" s="4" t="inlineStr">
+      <c r="T8" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U7" s="4" t="inlineStr">
+      <c r="U8" s="4" t="inlineStr">
         <is>
           <t>153.232.156.182</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>1254511136</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>滝澤　恵豪（タキザワ　ケイゴ）</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C9" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" s="1"/>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 21:18</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>滝澤　恵豪（タキザワ　ケイゴ）</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/YBl3Z2O3Ge47Wv16
 https://keigotakky3-eng.github.io/map01/</t>
         </is>
       </c>
-      <c r="J8" s="1"/>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M8" s="1"/>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O8" s="1"/>
-      <c r="P8" s="4" t="inlineStr">
+      <c r="J9" s="1"/>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M9" s="1"/>
+      <c r="N9" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O9" s="1"/>
+      <c r="P9" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q8" s="4" t="inlineStr">
+      <c r="Q9" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R8" s="4" t="inlineStr">
+      <c r="R9" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S8" s="4" t="inlineStr">
+      <c r="S9" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T8" s="4" t="inlineStr">
+      <c r="T9" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U8" s="4" t="inlineStr">
+      <c r="U9" s="4" t="inlineStr">
         <is>
           <t>222.6.232.21</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>1254511251</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>土屋　響輝（ツチヤ　ヒビキ）</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" s="1"/>
+      <c r="G10" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:22</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>土屋　響輝（ツチヤ　ヒビキ）</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Padlet URL
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/lkROZPpJDzrMZjMg
@@ -925,194 +1017,103 @@
 https://github.com/hibiki20060716/map01.git</t>
         </is>
       </c>
-      <c r="J9" s="1"/>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M9" s="1"/>
-      <c r="N9" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O9" s="1"/>
-      <c r="P9" s="4" t="inlineStr">
+      <c r="J10" s="1"/>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" s="1"/>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O10" s="1"/>
+      <c r="P10" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q9" s="4" t="inlineStr">
+      <c r="Q10" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R9" s="4" t="inlineStr">
+      <c r="R10" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 経済学部 経済学科 経済</t>
         </is>
       </c>
-      <c r="S9" s="4" t="inlineStr">
+      <c r="S10" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T9" s="4" t="inlineStr">
+      <c r="T10" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U9" s="4" t="inlineStr">
+      <c r="U10" s="4" t="inlineStr">
         <is>
           <t>61.23.189.153</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>1254511912</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>金澤　一華（カナザワ　イチカ）</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F10" s="1"/>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" s="1"/>
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 22:04</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>金澤　一華（カナザワ　イチカ）</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>https://a250989i-code.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/e9YpQNpzDj2lWxjM</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J11" s="4" t="inlineStr">
         <is>
           <t>元々南柏での空きコマを潰せる場所マップを作ろうと思っていましたが、今回の講義でみんなのサイトを見たときに音楽をつけたり、飛べるようにしたりできる面白いものを作りたいと思ってプロジェクトの内容を変えてしまいました。まだ私が自信を持って見せれるものではないので、サイトを開いたらもっと心躍るものを作りたいです。</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M10" s="1"/>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O10" s="1"/>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>2年</t>
-        </is>
-      </c>
-      <c r="Q10" s="4" t="inlineStr">
-        <is>
-          <t>3セメスタ</t>
-        </is>
-      </c>
-      <c r="R10" s="4" t="inlineStr">
-        <is>
-          <t>麗澤大学 経済学部 経済学科 経済</t>
-        </is>
-      </c>
-      <c r="S10" s="4" t="inlineStr">
-        <is>
-          <t>2025年度 春</t>
-        </is>
-      </c>
-      <c r="T10" s="4" t="inlineStr">
-        <is>
-          <t>進級</t>
-        </is>
-      </c>
-      <c r="U10" s="4" t="inlineStr">
-        <is>
-          <t>118.156.108.198</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>1254512085</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>宮城　大空（ミヤギ　ソラ）</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F11" s="1"/>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>2026/06/16 09:52</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>宮城　大空（ミヤギ　ソラ）</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>https://github.com/7p6nvbdgst-dev/map01.githttps://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/zV61Q6xkVYLbWO98</t>
-        </is>
-      </c>
-      <c r="J11" s="1"/>
       <c r="K11" s="4" t="inlineStr">
         <is>
           <t/>
@@ -1157,19 +1158,19 @@
       </c>
       <c r="U11" s="4" t="inlineStr">
         <is>
-          <t>153.169.20.190</t>
+          <t>118.156.108.198</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>1254512134</t>
+          <t>1254512085</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>荒井　聡（アライ　アキラ）</t>
+          <t>宮城　大空（ミヤギ　ソラ）</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1190,17 +1191,17 @@
       <c r="F12" s="1"/>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>2026/06/16 10:57</t>
+          <t>2026/06/16 09:52</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>荒井　聡（アライ　アキラ）</t>
+          <t>宮城　大空（ミヤギ　ソラ）</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>https://gis-araiakira.github.io/map01/</t>
+          <t>https://github.com/7p6nvbdgst-dev/map01.githttps://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/zV61Q6xkVYLbWO98</t>
         </is>
       </c>
       <c r="J12" s="1"/>
@@ -1248,19 +1249,19 @@
       </c>
       <c r="U12" s="4" t="inlineStr">
         <is>
-          <t>10.30.57.12</t>
+          <t>153.169.20.190</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>1254690352</t>
+          <t>1254512134</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+          <t>荒井　聡（アライ　アキラ）</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1281,199 +1282,290 @@
       <c r="F13" s="1"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
+          <t>2026/06/16 10:57</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>荒井　聡（アライ　アキラ）</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>https://gis-araiakira.github.io/map01/</t>
+        </is>
+      </c>
+      <c r="J13" s="1"/>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O13" s="1"/>
+      <c r="P13" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q13" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R13" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 経済学部 経済学科 経済</t>
+        </is>
+      </c>
+      <c r="S13" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T13" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U13" s="4" t="inlineStr">
+        <is>
+          <t>10.30.57.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>1254690352</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F14" s="1"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
           <t>2026/06/11 11:20</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>ＪＥＯＮ　ＹＵＢＥＥＮ（チョン　ユビン）</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2NvBGBZgP7
 https://jyb1472.github.io/map01/</t>
         </is>
       </c>
-      <c r="J13" s="1"/>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M13" s="1"/>
-      <c r="N13" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O13" s="1"/>
-      <c r="P13" s="4" t="inlineStr">
+      <c r="J14" s="1"/>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" s="1"/>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O14" s="1"/>
+      <c r="P14" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q13" s="4" t="inlineStr">
+      <c r="Q14" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R13" s="4" t="inlineStr">
+      <c r="R14" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際交流国際協力</t>
         </is>
       </c>
-      <c r="S13" s="4" t="inlineStr">
+      <c r="S14" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T13" s="4" t="inlineStr">
+      <c r="T14" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U13" s="4" t="inlineStr">
+      <c r="U14" s="4" t="inlineStr">
         <is>
           <t>10.30.50.131</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>1254690435</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F14" s="1"/>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 19:26</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H15" s="4" t="inlineStr">
         <is>
           <t>ＰＥＲＥＲＡ　ＭＥＶＥＮＳＴＥＥＶＥ（ペレラ　メブンスティーブ）</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I15" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿のURL: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/j40PQDYqXVweZvXB
 GitHub Pages のURL : https://nejihyugamsp.github.io/UNESCO-World-Map/</t>
         </is>
       </c>
-      <c r="J14" s="1"/>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M14" s="1"/>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O14" s="1"/>
-      <c r="P14" s="4" t="inlineStr">
+      <c r="J15" s="1"/>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M15" s="1"/>
+      <c r="N15" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O15" s="1"/>
+      <c r="P15" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q14" s="4" t="inlineStr">
+      <c r="Q15" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R14" s="4" t="inlineStr">
+      <c r="R15" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 国際学部 国際学科 国際社会</t>
         </is>
       </c>
-      <c r="S14" s="4" t="inlineStr">
+      <c r="S15" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T14" s="4" t="inlineStr">
+      <c r="T15" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U14" s="4" t="inlineStr">
+      <c r="U15" s="4" t="inlineStr">
         <is>
           <t>126.114.113.205</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>1254810059</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F16" s="1"/>
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:02</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>粟野　翔（アワノ　カケル）</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Padlet投稿
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/kxodWG2jDgRMZgP7
@@ -1481,1114 +1573,1023 @@
 https://awano-kakeru.github.io/map01/</t>
         </is>
       </c>
-      <c r="J15" s="1"/>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M15" s="1"/>
-      <c r="N15" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O15" s="1"/>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="J16" s="1"/>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M16" s="1"/>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O16" s="1"/>
+      <c r="P16" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q15" s="4" t="inlineStr">
+      <c r="Q16" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R15" s="4" t="inlineStr">
+      <c r="R16" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S15" s="4" t="inlineStr">
+      <c r="S16" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T15" s="4" t="inlineStr">
+      <c r="T16" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U15" s="4" t="inlineStr">
+      <c r="U16" s="4" t="inlineStr">
         <is>
           <t>10.30.25.13</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>1254810075</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F17" s="1"/>
+      <c r="G17" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 22:17</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr">
         <is>
           <t>石引　響（イシビキ　ヒビキ）</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Padlet:https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/e9YpQNpzDoXDWxjM
 GitHub Pages:https://a250818h-ai.github.io/map01/</t>
         </is>
       </c>
-      <c r="J16" s="1"/>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M16" s="1"/>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O16" s="1"/>
-      <c r="P16" s="4" t="inlineStr">
+      <c r="J17" s="1"/>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M17" s="1"/>
+      <c r="N17" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O17" s="1"/>
+      <c r="P17" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q16" s="4" t="inlineStr">
+      <c r="Q17" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R16" s="4" t="inlineStr">
+      <c r="R17" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S16" s="4" t="inlineStr">
+      <c r="S17" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T16" s="4" t="inlineStr">
+      <c r="T17" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U16" s="4" t="inlineStr">
+      <c r="U17" s="4" t="inlineStr">
         <is>
           <t>106.160.0.32</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>1254810124</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F18" s="1"/>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 23:49</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>江口　歩真（エグチ　アユマ）</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>https://ayuma-wp.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/x5A7aroMvBBxQwr6</t>
         </is>
       </c>
-      <c r="J17" s="1"/>
-      <c r="K17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M17" s="1"/>
-      <c r="N17" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O17" s="1"/>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="J18" s="1"/>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M18" s="1"/>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O18" s="1"/>
+      <c r="P18" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q17" s="4" t="inlineStr">
+      <c r="Q18" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R17" s="4" t="inlineStr">
+      <c r="R18" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S17" s="4" t="inlineStr">
+      <c r="S18" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T17" s="4" t="inlineStr">
+      <c r="T18" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U17" s="4" t="inlineStr">
+      <c r="U18" s="4" t="inlineStr">
         <is>
           <t>36.12.197.93</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>1254810140</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F18" s="1"/>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F19" s="1"/>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 06:47</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr">
         <is>
           <t>太田　和毅（オオタ　カズキ）</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjAKwnqa0OX
 https://kazu2856.github.io/fammap/
 https://github.com/kazu2856/fammap</t>
         </is>
       </c>
-      <c r="J18" s="1"/>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M18" s="1"/>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O18" s="1"/>
-      <c r="P18" s="4" t="inlineStr">
+      <c r="J19" s="1"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M19" s="1"/>
+      <c r="N19" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O19" s="1"/>
+      <c r="P19" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q18" s="4" t="inlineStr">
+      <c r="Q19" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R18" s="4" t="inlineStr">
+      <c r="R19" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S18" s="4" t="inlineStr">
+      <c r="S19" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T18" s="4" t="inlineStr">
+      <c r="T19" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U18" s="4" t="inlineStr">
+      <c r="U19" s="4" t="inlineStr">
         <is>
           <t>133.114.4.189</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>1254810166</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F20" s="1"/>
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:57</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>小川　史温（オガワ　シオン）</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>Padlet: https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/R7dXadN53qbeZ6bl
 git hub: a250827o-blip.github.io/map02/</t>
         </is>
       </c>
-      <c r="J19" s="1"/>
-      <c r="K19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M19" s="1"/>
-      <c r="N19" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O19" s="1"/>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="J20" s="1"/>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M20" s="1"/>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O20" s="1"/>
+      <c r="P20" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q19" s="4" t="inlineStr">
+      <c r="Q20" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R19" s="4" t="inlineStr">
+      <c r="R20" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S19" s="4" t="inlineStr">
+      <c r="S20" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T19" s="4" t="inlineStr">
+      <c r="T20" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U19" s="4" t="inlineStr">
+      <c r="U20" s="4" t="inlineStr">
         <is>
           <t>153.241.128.1</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>1254810174</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F20" s="1"/>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F21" s="1"/>
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:50</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H21" s="4" t="inlineStr">
         <is>
           <t>鬼塚　駿（オニツカ　シュン）</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/do3MQJwe0LnOZ15w
 https://shun-onitsuka.github.io/map01/</t>
         </is>
       </c>
-      <c r="J20" s="1"/>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M20" s="1"/>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O20" s="1"/>
-      <c r="P20" s="4" t="inlineStr">
+      <c r="J21" s="1"/>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O21" s="1"/>
+      <c r="P21" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q20" s="4" t="inlineStr">
+      <c r="Q21" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R20" s="4" t="inlineStr">
+      <c r="R21" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S20" s="4" t="inlineStr">
+      <c r="S21" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T20" s="4" t="inlineStr">
+      <c r="T21" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U20" s="4" t="inlineStr">
+      <c r="U21" s="4" t="inlineStr">
         <is>
           <t>59.132.16.22</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>1254810182</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B22" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C22" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D22" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="5" t="inlineStr">
         <is>
           <t>2026/06/09 16:14</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>柿木　奏太（カキノキ　ソウタ）</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I22" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/J24jalobBy6YW0A1
 https://github.com/a250829s-code/earth-map.git
 https://a250829s-code.github.io/earth-map/</t>
         </is>
       </c>
-      <c r="J21" s="1"/>
-      <c r="K21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M21" s="1"/>
-      <c r="N21" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O21" s="1"/>
-      <c r="P21" s="4" t="inlineStr">
+      <c r="J22" s="1"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M22" s="1"/>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O22" s="1"/>
+      <c r="P22" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q21" s="4" t="inlineStr">
+      <c r="Q22" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R21" s="4" t="inlineStr">
+      <c r="R22" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S21" s="4" t="inlineStr">
+      <c r="S22" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T21" s="4" t="inlineStr">
+      <c r="T22" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U21" s="4" t="inlineStr">
+      <c r="U22" s="4" t="inlineStr">
         <is>
           <t>10.30.60.247</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>1254810299</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F22" s="1"/>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F23" s="1"/>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 13:32</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H23" s="4" t="inlineStr">
         <is>
           <t>桑久保　陽平（クワクボ　ヨウヘイ）</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/AL83Wz7JPBnXa0Pg(padlet)
 https://1254810299.github.io/map01/(gitpages)</t>
         </is>
       </c>
-      <c r="J22" s="1"/>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M22" s="1"/>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O22" s="1"/>
-      <c r="P22" s="4" t="inlineStr">
+      <c r="J23" s="1"/>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M23" s="1"/>
+      <c r="N23" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O23" s="1"/>
+      <c r="P23" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q22" s="4" t="inlineStr">
+      <c r="Q23" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R22" s="4" t="inlineStr">
+      <c r="R23" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S22" s="4" t="inlineStr">
+      <c r="S23" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T22" s="4" t="inlineStr">
+      <c r="T23" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U22" s="4" t="inlineStr">
+      <c r="U23" s="4" t="inlineStr">
         <is>
           <t>10.30.25.6</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
         <is>
           <t>1254810372</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B24" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C24" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D24" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F23" s="1"/>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" s="1"/>
+      <c r="G24" s="5" t="inlineStr">
         <is>
           <t>2026/06/14 12:36</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>佐藤　陸（サトウ　リク）</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I24" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/XGyBQb1x2VmgaL6K 
 https://sari6641.github.io/map01/</t>
         </is>
       </c>
-      <c r="J23" s="1"/>
-      <c r="K23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M23" s="1"/>
-      <c r="N23" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O23" s="1"/>
-      <c r="P23" s="4" t="inlineStr">
+      <c r="J24" s="1"/>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M24" s="1"/>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O24" s="1"/>
+      <c r="P24" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q23" s="4" t="inlineStr">
+      <c r="Q24" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R23" s="4" t="inlineStr">
+      <c r="R24" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S23" s="4" t="inlineStr">
+      <c r="S24" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T23" s="4" t="inlineStr">
+      <c r="T24" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U23" s="4" t="inlineStr">
+      <c r="U24" s="4" t="inlineStr">
         <is>
           <t>106.128.107.23</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>1254810405</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D25" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="1"/>
+      <c r="G25" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:52</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H25" s="4" t="inlineStr">
         <is>
           <t>柴田　尚槻（シバタ　ナオキ）</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Xb8YaLpw5XlJayn1
 https://sibaba615.github.io/map1/
 https://github.com/sibaba615/map1</t>
         </is>
       </c>
-      <c r="J24" s="1"/>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M24" s="1"/>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O24" s="1"/>
-      <c r="P24" s="4" t="inlineStr">
+      <c r="J25" s="1"/>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M25" s="1"/>
+      <c r="N25" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O25" s="1"/>
+      <c r="P25" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q24" s="4" t="inlineStr">
+      <c r="Q25" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R24" s="4" t="inlineStr">
+      <c r="R25" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S24" s="4" t="inlineStr">
+      <c r="S25" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T24" s="4" t="inlineStr">
+      <c r="T25" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U24" s="4" t="inlineStr">
+      <c r="U25" s="4" t="inlineStr">
         <is>
           <t>219.104.130.164</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>1254810413</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B26" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F26" s="1"/>
+      <c r="G26" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 00:07</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>島田　晟（シマダ　ジョウ）</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I26" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/yEPVZkoXldopZb0Y
 https://joe-0711.github.io/map01/
 https://github.com/joe-0711/map01</t>
         </is>
       </c>
-      <c r="J25" s="1"/>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M25" s="1"/>
-      <c r="N25" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O25" s="1"/>
-      <c r="P25" s="4" t="inlineStr">
+      <c r="J26" s="1"/>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M26" s="1"/>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O26" s="1"/>
+      <c r="P26" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q25" s="4" t="inlineStr">
+      <c r="Q26" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R25" s="4" t="inlineStr">
+      <c r="R26" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S25" s="4" t="inlineStr">
+      <c r="S26" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T25" s="4" t="inlineStr">
+      <c r="T26" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U25" s="4" t="inlineStr">
+      <c r="U26" s="4" t="inlineStr">
         <is>
           <t>60.93.159.60</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>1254810512</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F26" s="1"/>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F27" s="1"/>
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:11</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H27" s="4" t="inlineStr">
         <is>
           <t>竹田　圭冴（タケタ　ケイゴ）</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>https://taketaago.github.io/map01/
 https://github.com/taketaago/map01
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/L8KjW9vyykk2aJbv</t>
         </is>
       </c>
-      <c r="J26" s="1"/>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M26" s="1"/>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O26" s="1"/>
-      <c r="P26" s="4" t="inlineStr">
-        <is>
-          <t>2年</t>
-        </is>
-      </c>
-      <c r="Q26" s="4" t="inlineStr">
-        <is>
-          <t>3セメスタ</t>
-        </is>
-      </c>
-      <c r="R26" s="4" t="inlineStr">
-        <is>
-          <t>麗澤大学 工学部 工学科 情報システム工学</t>
-        </is>
-      </c>
-      <c r="S26" s="4" t="inlineStr">
-        <is>
-          <t>2025年度 春</t>
-        </is>
-      </c>
-      <c r="T26" s="4" t="inlineStr">
-        <is>
-          <t>進級</t>
-        </is>
-      </c>
-      <c r="U26" s="4" t="inlineStr">
-        <is>
-          <t>150.91.180.64</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>1254810562</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>○</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F27" s="1"/>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>2026/06/10 19:53</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t>永野　虎太郎（ナガノ　コタロウ）</t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
-        </is>
-      </c>
       <c r="J27" s="1"/>
       <c r="K27" s="4" t="inlineStr">
         <is>
@@ -2634,19 +2635,19 @@
       </c>
       <c r="U27" s="4" t="inlineStr">
         <is>
-          <t>1.115.90.218</t>
+          <t>150.91.180.64</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>1254810588</t>
+          <t>1254810562</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>野村　隆介（ノムラ　リュウスケ）</t>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2667,801 +2668,892 @@
       <c r="F28" s="1"/>
       <c r="G28" s="5" t="inlineStr">
         <is>
+          <t>2026/06/10 19:53</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>永野　虎太郎（ナガノ　コタロウ）</t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>まだ発表内容が決まってないためまだ目星がついていない次の時に名前プロジェクトを話し合う予定</t>
+        </is>
+      </c>
+      <c r="J28" s="1"/>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M28" s="1"/>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>2年</t>
+        </is>
+      </c>
+      <c r="Q28" s="4" t="inlineStr">
+        <is>
+          <t>3セメスタ</t>
+        </is>
+      </c>
+      <c r="R28" s="4" t="inlineStr">
+        <is>
+          <t>麗澤大学 工学部 工学科 情報システム工学</t>
+        </is>
+      </c>
+      <c r="S28" s="4" t="inlineStr">
+        <is>
+          <t>2025年度 春</t>
+        </is>
+      </c>
+      <c r="T28" s="4" t="inlineStr">
+        <is>
+          <t>進級</t>
+        </is>
+      </c>
+      <c r="U28" s="4" t="inlineStr">
+        <is>
+          <t>1.115.90.218</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>1254810588</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>野村　隆介（ノムラ　リュウスケ）</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F29" s="1"/>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
           <t>2026/06/13 13:52</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>野村　隆介（ノムラ　リュウスケ）</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mDRxWBq0x4rOZjb1
 https://nomuraryuusuke.github.io/map----/</t>
         </is>
       </c>
-      <c r="J28" s="1"/>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M28" s="1"/>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O28" s="1"/>
-      <c r="P28" s="4" t="inlineStr">
+      <c r="J29" s="1"/>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M29" s="1"/>
+      <c r="N29" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O29" s="1"/>
+      <c r="P29" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q28" s="4" t="inlineStr">
+      <c r="Q29" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R28" s="4" t="inlineStr">
+      <c r="R29" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S28" s="4" t="inlineStr">
+      <c r="S29" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T28" s="4" t="inlineStr">
+      <c r="T29" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U28" s="4" t="inlineStr">
+      <c r="U29" s="4" t="inlineStr">
         <is>
           <t>118.241.60.18</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>1254810736</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F29" s="1"/>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F30" s="1"/>
+      <c r="G30" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 13:34</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>三浦　和道（ミウラ　カズミチ）</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I30" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/jpoxajk68LqOQbPE
 https://yuu08080.github.io/map01/</t>
         </is>
       </c>
-      <c r="J29" s="1"/>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M29" s="1"/>
-      <c r="N29" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O29" s="1"/>
-      <c r="P29" s="4" t="inlineStr">
+      <c r="J30" s="1"/>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M30" s="1"/>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O30" s="1"/>
+      <c r="P30" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q29" s="4" t="inlineStr">
+      <c r="Q30" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R29" s="4" t="inlineStr">
+      <c r="R30" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S29" s="4" t="inlineStr">
+      <c r="S30" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T29" s="4" t="inlineStr">
+      <c r="T30" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U29" s="4" t="inlineStr">
+      <c r="U30" s="4" t="inlineStr">
         <is>
           <t>10.30.59.77</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>1254810794</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>桃井　優（モモイ　ユウ）</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F30" s="1"/>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F31" s="1"/>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 10:59</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H31" s="4" t="inlineStr">
         <is>
           <t>桃井　優（モモイ　ユウ）</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I31" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/j40PQDYDoE3XZvXB
 https://a250890y-cmd.github.io/memory_map_web/</t>
         </is>
       </c>
-      <c r="J30" s="1"/>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M30" s="1"/>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O30" s="1"/>
-      <c r="P30" s="4" t="inlineStr">
+      <c r="J31" s="1"/>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M31" s="1"/>
+      <c r="N31" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O31" s="1"/>
+      <c r="P31" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q30" s="4" t="inlineStr">
+      <c r="Q31" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R30" s="4" t="inlineStr">
+      <c r="R31" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S30" s="4" t="inlineStr">
+      <c r="S31" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T30" s="4" t="inlineStr">
+      <c r="T31" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U30" s="4" t="inlineStr">
+      <c r="U31" s="4" t="inlineStr">
         <is>
           <t>10.30.56.176</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>1254810801</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D32" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F31" s="1"/>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F32" s="1"/>
+      <c r="G32" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 01:23</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>森本　颯太（モリモト　ソウタ）</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/NvylWEjABEY3a0OX
  https://souta-1213.github.io/map01/</t>
         </is>
       </c>
-      <c r="J31" s="1"/>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M31" s="1"/>
-      <c r="N31" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O31" s="1"/>
-      <c r="P31" s="4" t="inlineStr">
+      <c r="J32" s="1"/>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M32" s="1"/>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O32" s="1"/>
+      <c r="P32" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q31" s="4" t="inlineStr">
+      <c r="Q32" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R31" s="4" t="inlineStr">
+      <c r="R32" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S31" s="4" t="inlineStr">
+      <c r="S32" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T31" s="4" t="inlineStr">
+      <c r="T32" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U31" s="4" t="inlineStr">
+      <c r="U32" s="4" t="inlineStr">
         <is>
           <t>126.249.152.193</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>1254810827</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D33" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F32" s="1"/>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F33" s="1"/>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 09:14</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H33" s="4" t="inlineStr">
         <is>
           <t>八重樫　旺樹（ヤエガシ　ヒロキ）</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/LNV1Q7y77JrrWmq3
 https://yaegashi0314.github.io/map001/</t>
         </is>
       </c>
-      <c r="J32" s="1"/>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M32" s="1"/>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O32" s="1"/>
-      <c r="P32" s="4" t="inlineStr">
+      <c r="J33" s="1"/>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M33" s="1"/>
+      <c r="N33" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O33" s="1"/>
+      <c r="P33" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q32" s="4" t="inlineStr">
+      <c r="Q33" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R32" s="4" t="inlineStr">
+      <c r="R33" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S32" s="4" t="inlineStr">
+      <c r="S33" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T32" s="4" t="inlineStr">
+      <c r="T33" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U32" s="4" t="inlineStr">
+      <c r="U33" s="4" t="inlineStr">
         <is>
           <t>118.83.190.225</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>1254810926</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B34" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F33" s="1"/>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F34" s="1"/>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 08:55</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>吉田　爽二（ヨシダ　ソウジ）</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I34" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/mlNDZ3OGGDrqZznG
 https://github.com/a250903y-gif/a250903y-gif.github.io.git</t>
         </is>
       </c>
-      <c r="J33" s="1"/>
-      <c r="K33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M33" s="1"/>
-      <c r="N33" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O33" s="1"/>
-      <c r="P33" s="4" t="inlineStr">
+      <c r="J34" s="1"/>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M34" s="1"/>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O34" s="1"/>
+      <c r="P34" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q33" s="4" t="inlineStr">
+      <c r="Q34" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R33" s="4" t="inlineStr">
+      <c r="R34" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S33" s="4" t="inlineStr">
+      <c r="S34" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T33" s="4" t="inlineStr">
+      <c r="T34" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U33" s="4" t="inlineStr">
+      <c r="U34" s="4" t="inlineStr">
         <is>
           <t>116.82.97.244</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>1254810976</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B35" s="4" t="inlineStr">
         <is>
           <t>坂本　快（サカモト　カイ）</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F34" s="1"/>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F35" s="1"/>
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>2026/06/16 10:39</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H35" s="4" t="inlineStr">
         <is>
           <t>坂本　快（サカモト　カイ）</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I35" s="4" t="inlineStr">
         <is>
           <t>https://kai-sakamoto.github.io/map01/
 https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/dMA1W85Rz97Xa4OV</t>
         </is>
       </c>
-      <c r="J34" s="1"/>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M34" s="1"/>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O34" s="1"/>
-      <c r="P34" s="4" t="inlineStr">
+      <c r="J35" s="1"/>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M35" s="1"/>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O35" s="1"/>
+      <c r="P35" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q34" s="4" t="inlineStr">
+      <c r="Q35" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R34" s="4" t="inlineStr">
+      <c r="R35" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S34" s="4" t="inlineStr">
+      <c r="S35" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T34" s="4" t="inlineStr">
+      <c r="T35" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U34" s="4" t="inlineStr">
+      <c r="U35" s="4" t="inlineStr">
         <is>
           <t>10.30.25.100</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>1254810992</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F35" s="1"/>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="5" t="inlineStr">
         <is>
           <t>2026/06/12 14:01</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>ＭＯＮＴＥＬＬＡ　ＥＤＷＩＮ（モンテッラ　エドウィン）</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/Ae2Ravoe2PpOQnz4
 https://github.com/edwin379/train
 https://train-5dwy.onrender.com/</t>
         </is>
       </c>
-      <c r="J35" s="1"/>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M35" s="1"/>
-      <c r="N35" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O35" s="1"/>
-      <c r="P35" s="4" t="inlineStr">
+      <c r="J36" s="1"/>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M36" s="1"/>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O36" s="1"/>
+      <c r="P36" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q35" s="4" t="inlineStr">
+      <c r="Q36" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R35" s="4" t="inlineStr">
+      <c r="R36" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 情報システム工学</t>
         </is>
       </c>
-      <c r="S35" s="4" t="inlineStr">
+      <c r="S36" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T35" s="4" t="inlineStr">
+      <c r="T36" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U35" s="4" t="inlineStr">
+      <c r="U36" s="4" t="inlineStr">
         <is>
           <t>10.30.56.85</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>1254820222</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>○</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D37" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F36" s="1"/>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F37" s="1"/>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>2026/06/15 20:09</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H37" s="4" t="inlineStr">
         <is>
           <t>神戸　宗一郎（カンベ　ソウイチロウ）</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>https://padlet.com/tsasao/26-1-reitaku-gis-acbkafzbx0kp4mu0/wish/4b3zaMpVDXA9W2j7
 https://github.com/a250927s-create/HIPHOPMAP.git</t>
         </is>
       </c>
-      <c r="J36" s="1"/>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M36" s="1"/>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O36" s="1"/>
-      <c r="P36" s="4" t="inlineStr">
+      <c r="J37" s="1"/>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M37" s="1"/>
+      <c r="N37" s="4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O37" s="1"/>
+      <c r="P37" s="4" t="inlineStr">
         <is>
           <t>2年</t>
         </is>
       </c>
-      <c r="Q36" s="4" t="inlineStr">
+      <c r="Q37" s="4" t="inlineStr">
         <is>
           <t>3セメスタ</t>
         </is>
       </c>
-      <c r="R36" s="4" t="inlineStr">
+      <c r="R37" s="4" t="inlineStr">
         <is>
           <t>麗澤大学 工学部 工学科 ロボティクス</t>
         </is>
       </c>
-      <c r="S36" s="4" t="inlineStr">
+      <c r="S37" s="4" t="inlineStr">
         <is>
           <t>2025年度 春</t>
         </is>
       </c>
-      <c r="T36" s="4" t="inlineStr">
+      <c r="T37" s="4" t="inlineStr">
         <is>
           <t>進級</t>
         </is>
       </c>
-      <c r="U36" s="4" t="inlineStr">
+      <c r="U37" s="4" t="inlineStr">
         <is>
           <t>10.30.48.85</t>
         </is>

</xml_diff>